<commit_message>
Suskaičiuoti greičiai iki greičių vidurkio
</commit_message>
<xml_diff>
--- a/PVZ2.xlsx
+++ b/PVZ2.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="147" documentId="8_{8FD3B17B-922A-42A3-879B-A575A223ADA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D4044E6-60E2-4BF7-BDD4-4F820AD5D73A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="2" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="1" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Compatibility Report" sheetId="4" state="hidden" r:id="rId1"/>
@@ -2658,14 +2658,122 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="29" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2675,115 +2783,7 @@
     <xf numFmtId="0" fontId="10" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="29" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -3283,31 +3283,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="D3" s="262" t="s">
+      <c r="D3" s="264" t="s">
         <v>102</v>
       </c>
-      <c r="E3" s="262"/>
-      <c r="F3" s="262"/>
-      <c r="G3" s="262"/>
-      <c r="H3" s="262"/>
-      <c r="I3" s="262"/>
-      <c r="J3" s="262"/>
-      <c r="K3" s="262"/>
-      <c r="L3" s="262"/>
-      <c r="M3" s="262"/>
-      <c r="N3" s="262"/>
-      <c r="O3" s="262"/>
-      <c r="P3" s="262"/>
-      <c r="Q3" s="262"/>
-      <c r="R3" s="262"/>
-      <c r="S3" s="262"/>
-      <c r="T3" s="262"/>
-      <c r="U3" s="262"/>
-      <c r="V3" s="262"/>
-      <c r="W3" s="262"/>
-      <c r="X3" s="262"/>
-      <c r="Y3" s="262"/>
-      <c r="Z3" s="262"/>
+      <c r="E3" s="264"/>
+      <c r="F3" s="264"/>
+      <c r="G3" s="264"/>
+      <c r="H3" s="264"/>
+      <c r="I3" s="264"/>
+      <c r="J3" s="264"/>
+      <c r="K3" s="264"/>
+      <c r="L3" s="264"/>
+      <c r="M3" s="264"/>
+      <c r="N3" s="264"/>
+      <c r="O3" s="264"/>
+      <c r="P3" s="264"/>
+      <c r="Q3" s="264"/>
+      <c r="R3" s="264"/>
+      <c r="S3" s="264"/>
+      <c r="T3" s="264"/>
+      <c r="U3" s="264"/>
+      <c r="V3" s="264"/>
+      <c r="W3" s="264"/>
+      <c r="X3" s="264"/>
+      <c r="Y3" s="264"/>
+      <c r="Z3" s="264"/>
     </row>
     <row r="5" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
@@ -3396,13 +3396,13 @@
       </c>
     </row>
     <row r="6" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="263" t="s">
+      <c r="A6" s="265" t="s">
         <v>138</v>
       </c>
-      <c r="B6" s="266" t="s">
+      <c r="B6" s="268" t="s">
         <v>139</v>
       </c>
-      <c r="C6" s="267" t="s">
+      <c r="C6" s="269" t="s">
         <v>140</v>
       </c>
       <c r="D6" s="127">
@@ -3488,14 +3488,14 @@
         <f>Aerodinamika!G23</f>
         <v>1.2973599999999998</v>
       </c>
-      <c r="AB6" s="260" t="s">
+      <c r="AB6" s="262" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A7" s="264"/>
-      <c r="B7" s="264"/>
-      <c r="C7" s="268"/>
+      <c r="A7" s="266"/>
+      <c r="B7" s="266"/>
+      <c r="C7" s="270"/>
       <c r="D7" s="127">
         <v>19</v>
       </c>
@@ -3575,12 +3575,12 @@
         <f>O6*X7</f>
         <v>0.34740732161375365</v>
       </c>
-      <c r="AB7" s="261"/>
+      <c r="AB7" s="263"/>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A8" s="264"/>
-      <c r="B8" s="264"/>
-      <c r="C8" s="268"/>
+      <c r="A8" s="266"/>
+      <c r="B8" s="266"/>
+      <c r="C8" s="270"/>
       <c r="D8" s="254">
         <v>33</v>
       </c>
@@ -3626,9 +3626,9 @@
       <c r="S8" s="126"/>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A9" s="264"/>
-      <c r="B9" s="264"/>
-      <c r="C9" s="268"/>
+      <c r="A9" s="266"/>
+      <c r="B9" s="266"/>
+      <c r="C9" s="270"/>
       <c r="D9" s="127">
         <v>48</v>
       </c>
@@ -3678,9 +3678,9 @@
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A10" s="264"/>
-      <c r="B10" s="264"/>
-      <c r="C10" s="268"/>
+      <c r="A10" s="266"/>
+      <c r="B10" s="266"/>
+      <c r="C10" s="270"/>
       <c r="D10" s="127">
         <v>65</v>
       </c>
@@ -3719,9 +3719,9 @@
       <c r="N10" s="179"/>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A11" s="264"/>
-      <c r="B11" s="264"/>
-      <c r="C11" s="268"/>
+      <c r="A11" s="266"/>
+      <c r="B11" s="266"/>
+      <c r="C11" s="270"/>
       <c r="D11" s="127">
         <v>85</v>
       </c>
@@ -3760,9 +3760,9 @@
       <c r="N11" s="179"/>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A12" s="264"/>
-      <c r="B12" s="264"/>
-      <c r="C12" s="268"/>
+      <c r="A12" s="266"/>
+      <c r="B12" s="266"/>
+      <c r="C12" s="270"/>
       <c r="D12" s="127">
         <v>108</v>
       </c>
@@ -3801,9 +3801,9 @@
       <c r="N12" s="179"/>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A13" s="264"/>
-      <c r="B13" s="264"/>
-      <c r="C13" s="268"/>
+      <c r="A13" s="266"/>
+      <c r="B13" s="266"/>
+      <c r="C13" s="270"/>
       <c r="D13" s="127">
         <v>140</v>
       </c>
@@ -3843,9 +3843,9 @@
       <c r="O13" s="124"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A14" s="264"/>
-      <c r="B14" s="264"/>
-      <c r="C14" s="268"/>
+      <c r="A14" s="266"/>
+      <c r="B14" s="266"/>
+      <c r="C14" s="270"/>
       <c r="D14" s="127">
         <v>200</v>
       </c>
@@ -3888,9 +3888,9 @@
       <c r="U14" s="37"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A15" s="264"/>
-      <c r="B15" s="264"/>
-      <c r="C15" s="268"/>
+      <c r="A15" s="266"/>
+      <c r="B15" s="266"/>
+      <c r="C15" s="270"/>
       <c r="D15" s="127">
         <v>260</v>
       </c>
@@ -3933,9 +3933,9 @@
       <c r="U15" s="37"/>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A16" s="264"/>
-      <c r="B16" s="264"/>
-      <c r="C16" s="268"/>
+      <c r="A16" s="266"/>
+      <c r="B16" s="266"/>
+      <c r="C16" s="270"/>
       <c r="D16" s="127">
         <v>292</v>
       </c>
@@ -3978,9 +3978,9 @@
       <c r="U16" s="37"/>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A17" s="264"/>
-      <c r="B17" s="264"/>
-      <c r="C17" s="268"/>
+      <c r="A17" s="266"/>
+      <c r="B17" s="266"/>
+      <c r="C17" s="270"/>
       <c r="D17" s="127">
         <v>315</v>
       </c>
@@ -4023,9 +4023,9 @@
       <c r="U17" s="37"/>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A18" s="264"/>
-      <c r="B18" s="264"/>
-      <c r="C18" s="268"/>
+      <c r="A18" s="266"/>
+      <c r="B18" s="266"/>
+      <c r="C18" s="270"/>
       <c r="D18" s="127">
         <v>335</v>
       </c>
@@ -4068,9 +4068,9 @@
       <c r="U18" s="37"/>
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A19" s="264"/>
-      <c r="B19" s="264"/>
-      <c r="C19" s="268"/>
+      <c r="A19" s="266"/>
+      <c r="B19" s="266"/>
+      <c r="C19" s="270"/>
       <c r="D19" s="127">
         <v>352</v>
       </c>
@@ -4113,9 +4113,9 @@
       <c r="U19" s="37"/>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A20" s="264"/>
-      <c r="B20" s="264"/>
-      <c r="C20" s="268"/>
+      <c r="A20" s="266"/>
+      <c r="B20" s="266"/>
+      <c r="C20" s="270"/>
       <c r="D20" s="127">
         <v>367</v>
       </c>
@@ -4158,9 +4158,9 @@
       <c r="U20" s="37"/>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A21" s="264"/>
-      <c r="B21" s="264"/>
-      <c r="C21" s="268"/>
+      <c r="A21" s="266"/>
+      <c r="B21" s="266"/>
+      <c r="C21" s="270"/>
       <c r="D21" s="127">
         <v>381</v>
       </c>
@@ -4203,9 +4203,9 @@
       <c r="U21" s="37"/>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A22" s="265"/>
-      <c r="B22" s="265"/>
-      <c r="C22" s="269"/>
+      <c r="A22" s="267"/>
+      <c r="B22" s="267"/>
+      <c r="C22" s="271"/>
       <c r="D22" s="127">
         <v>394</v>
       </c>
@@ -4309,11 +4309,11 @@
         <v>0</v>
       </c>
       <c r="N24" s="69"/>
-      <c r="O24" s="270" t="s">
+      <c r="O24" s="272" t="s">
         <v>127</v>
       </c>
-      <c r="P24" s="271"/>
-      <c r="Q24" s="271"/>
+      <c r="P24" s="273"/>
+      <c r="Q24" s="273"/>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="157"/>
@@ -4348,30 +4348,30 @@
       <c r="A28" s="157"/>
       <c r="B28" s="157"/>
       <c r="C28" s="157"/>
-      <c r="D28" s="272" t="s">
+      <c r="D28" s="274" t="s">
         <v>129</v>
       </c>
-      <c r="E28" s="262"/>
-      <c r="F28" s="262"/>
-      <c r="G28" s="262"/>
-      <c r="H28" s="262"/>
-      <c r="I28" s="262"/>
-      <c r="J28" s="262"/>
-      <c r="K28" s="262"/>
-      <c r="L28" s="262"/>
-      <c r="M28" s="262"/>
-      <c r="N28" s="262"/>
-      <c r="O28" s="262"/>
-      <c r="P28" s="262"/>
-      <c r="Q28" s="262"/>
-      <c r="R28" s="262"/>
-      <c r="S28" s="262"/>
-      <c r="T28" s="262"/>
-      <c r="U28" s="262"/>
-      <c r="V28" s="262"/>
-      <c r="W28" s="262"/>
-      <c r="X28" s="262"/>
-      <c r="Y28" s="262"/>
+      <c r="E28" s="264"/>
+      <c r="F28" s="264"/>
+      <c r="G28" s="264"/>
+      <c r="H28" s="264"/>
+      <c r="I28" s="264"/>
+      <c r="J28" s="264"/>
+      <c r="K28" s="264"/>
+      <c r="L28" s="264"/>
+      <c r="M28" s="264"/>
+      <c r="N28" s="264"/>
+      <c r="O28" s="264"/>
+      <c r="P28" s="264"/>
+      <c r="Q28" s="264"/>
+      <c r="R28" s="264"/>
+      <c r="S28" s="264"/>
+      <c r="T28" s="264"/>
+      <c r="U28" s="264"/>
+      <c r="V28" s="264"/>
+      <c r="W28" s="264"/>
+      <c r="X28" s="264"/>
+      <c r="Y28" s="264"/>
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="157"/>
@@ -4476,9 +4476,9 @@
       </c>
     </row>
     <row r="31" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="273"/>
-      <c r="B31" s="273"/>
-      <c r="C31" s="273"/>
+      <c r="A31" s="275"/>
+      <c r="B31" s="275"/>
+      <c r="C31" s="275"/>
       <c r="D31" s="127">
         <v>6</v>
       </c>
@@ -4556,12 +4556,12 @@
         <f>Aerodinamika!G23</f>
         <v>1.2973599999999998</v>
       </c>
-      <c r="AB31" s="260"/>
+      <c r="AB31" s="262"/>
     </row>
     <row r="32" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A32" s="274"/>
-      <c r="B32" s="274"/>
-      <c r="C32" s="274"/>
+      <c r="A32" s="276"/>
+      <c r="B32" s="276"/>
+      <c r="C32" s="276"/>
       <c r="D32" s="127">
         <v>19</v>
       </c>
@@ -4632,12 +4632,12 @@
         <f>O31*X32</f>
         <v>0.34740732161375365</v>
       </c>
-      <c r="AB32" s="261"/>
+      <c r="AB32" s="263"/>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A33" s="274"/>
-      <c r="B33" s="274"/>
-      <c r="C33" s="274"/>
+      <c r="A33" s="276"/>
+      <c r="B33" s="276"/>
+      <c r="C33" s="276"/>
       <c r="D33" s="254">
         <v>33</v>
       </c>
@@ -4674,9 +4674,9 @@
       <c r="S33" s="126"/>
     </row>
     <row r="34" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A34" s="274"/>
-      <c r="B34" s="274"/>
-      <c r="C34" s="274"/>
+      <c r="A34" s="276"/>
+      <c r="B34" s="276"/>
+      <c r="C34" s="276"/>
       <c r="D34" s="127">
         <v>48</v>
       </c>
@@ -4717,9 +4717,9 @@
       </c>
     </row>
     <row r="35" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A35" s="274"/>
-      <c r="B35" s="274"/>
-      <c r="C35" s="274"/>
+      <c r="A35" s="276"/>
+      <c r="B35" s="276"/>
+      <c r="C35" s="276"/>
       <c r="D35" s="127">
         <v>65</v>
       </c>
@@ -4749,9 +4749,9 @@
       <c r="N35" s="133"/>
     </row>
     <row r="36" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A36" s="274"/>
-      <c r="B36" s="274"/>
-      <c r="C36" s="274"/>
+      <c r="A36" s="276"/>
+      <c r="B36" s="276"/>
+      <c r="C36" s="276"/>
       <c r="D36" s="127">
         <v>85</v>
       </c>
@@ -4781,9 +4781,9 @@
       <c r="N36" s="133"/>
     </row>
     <row r="37" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A37" s="274"/>
-      <c r="B37" s="274"/>
-      <c r="C37" s="274"/>
+      <c r="A37" s="276"/>
+      <c r="B37" s="276"/>
+      <c r="C37" s="276"/>
       <c r="D37" s="127">
         <v>108</v>
       </c>
@@ -4813,9 +4813,9 @@
       <c r="N37" s="133"/>
     </row>
     <row r="38" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A38" s="274"/>
-      <c r="B38" s="274"/>
-      <c r="C38" s="274"/>
+      <c r="A38" s="276"/>
+      <c r="B38" s="276"/>
+      <c r="C38" s="276"/>
       <c r="D38" s="127">
         <v>140</v>
       </c>
@@ -4846,9 +4846,9 @@
       <c r="O38" s="124"/>
     </row>
     <row r="39" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A39" s="274"/>
-      <c r="B39" s="274"/>
-      <c r="C39" s="274"/>
+      <c r="A39" s="276"/>
+      <c r="B39" s="276"/>
+      <c r="C39" s="276"/>
       <c r="D39" s="127">
         <v>200</v>
       </c>
@@ -4882,9 +4882,9 @@
       <c r="U39" s="37"/>
     </row>
     <row r="40" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A40" s="274"/>
-      <c r="B40" s="274"/>
-      <c r="C40" s="274"/>
+      <c r="A40" s="276"/>
+      <c r="B40" s="276"/>
+      <c r="C40" s="276"/>
       <c r="D40" s="127">
         <v>260</v>
       </c>
@@ -4914,9 +4914,9 @@
       <c r="N40" s="127"/>
     </row>
     <row r="41" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A41" s="274"/>
-      <c r="B41" s="274"/>
-      <c r="C41" s="274"/>
+      <c r="A41" s="276"/>
+      <c r="B41" s="276"/>
+      <c r="C41" s="276"/>
       <c r="D41" s="127">
         <v>292</v>
       </c>
@@ -4946,9 +4946,9 @@
       <c r="N41" s="127"/>
     </row>
     <row r="42" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A42" s="274"/>
-      <c r="B42" s="274"/>
-      <c r="C42" s="274"/>
+      <c r="A42" s="276"/>
+      <c r="B42" s="276"/>
+      <c r="C42" s="276"/>
       <c r="D42" s="127">
         <v>315</v>
       </c>
@@ -4978,9 +4978,9 @@
       <c r="N42" s="127"/>
     </row>
     <row r="43" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A43" s="274"/>
-      <c r="B43" s="274"/>
-      <c r="C43" s="274"/>
+      <c r="A43" s="276"/>
+      <c r="B43" s="276"/>
+      <c r="C43" s="276"/>
       <c r="D43" s="127">
         <v>335</v>
       </c>
@@ -5010,9 +5010,9 @@
       <c r="N43" s="127"/>
     </row>
     <row r="44" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A44" s="274"/>
-      <c r="B44" s="274"/>
-      <c r="C44" s="274"/>
+      <c r="A44" s="276"/>
+      <c r="B44" s="276"/>
+      <c r="C44" s="276"/>
       <c r="D44" s="127">
         <v>352</v>
       </c>
@@ -5042,9 +5042,9 @@
       <c r="N44" s="127"/>
     </row>
     <row r="45" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A45" s="274"/>
-      <c r="B45" s="274"/>
-      <c r="C45" s="274"/>
+      <c r="A45" s="276"/>
+      <c r="B45" s="276"/>
+      <c r="C45" s="276"/>
       <c r="D45" s="127">
         <v>367</v>
       </c>
@@ -5074,9 +5074,9 @@
       <c r="N45" s="127"/>
     </row>
     <row r="46" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A46" s="274"/>
-      <c r="B46" s="274"/>
-      <c r="C46" s="274"/>
+      <c r="A46" s="276"/>
+      <c r="B46" s="276"/>
+      <c r="C46" s="276"/>
       <c r="D46" s="127">
         <v>381</v>
       </c>
@@ -5106,9 +5106,9 @@
       <c r="N46" s="127"/>
     </row>
     <row r="47" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A47" s="275"/>
-      <c r="B47" s="275"/>
-      <c r="C47" s="275"/>
+      <c r="A47" s="277"/>
+      <c r="B47" s="277"/>
+      <c r="C47" s="277"/>
       <c r="D47" s="127">
         <v>394</v>
       </c>
@@ -5196,18 +5196,18 @@
       <c r="I2" s="10"/>
     </row>
     <row r="3" spans="1:12" ht="15" x14ac:dyDescent="0.3">
-      <c r="A3" s="276" t="s">
+      <c r="A3" s="255" t="s">
         <v>101</v>
       </c>
-      <c r="B3" s="276"/>
-      <c r="C3" s="276"/>
-      <c r="D3" s="276"/>
-      <c r="E3" s="276"/>
-      <c r="F3" s="276"/>
-      <c r="G3" s="276"/>
-      <c r="H3" s="276"/>
-      <c r="I3" s="276"/>
-      <c r="J3" s="276"/>
+      <c r="B3" s="255"/>
+      <c r="C3" s="255"/>
+      <c r="D3" s="255"/>
+      <c r="E3" s="255"/>
+      <c r="F3" s="255"/>
+      <c r="G3" s="255"/>
+      <c r="H3" s="255"/>
+      <c r="I3" s="255"/>
+      <c r="J3" s="255"/>
     </row>
     <row r="4" spans="1:12" ht="14" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
@@ -5354,46 +5354,46 @@
       <c r="L10" s="44"/>
     </row>
     <row r="11" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H11" s="277" t="s">
+      <c r="H11" s="256" t="s">
         <v>28</v>
       </c>
-      <c r="I11" s="280" t="s">
+      <c r="I11" s="259" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H12" s="278"/>
-      <c r="I12" s="281"/>
+      <c r="H12" s="257"/>
+      <c r="I12" s="260"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H13" s="278"/>
-      <c r="I13" s="281"/>
+      <c r="H13" s="257"/>
+      <c r="I13" s="260"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H14" s="278"/>
-      <c r="I14" s="281"/>
+      <c r="H14" s="257"/>
+      <c r="I14" s="260"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H15" s="278"/>
-      <c r="I15" s="281"/>
+      <c r="H15" s="257"/>
+      <c r="I15" s="260"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H16" s="278"/>
-      <c r="I16" s="281"/>
+      <c r="H16" s="257"/>
+      <c r="I16" s="260"/>
     </row>
     <row r="17" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H17" s="278"/>
-      <c r="I17" s="281"/>
+      <c r="H17" s="257"/>
+      <c r="I17" s="260"/>
     </row>
     <row r="18" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H18" s="279"/>
-      <c r="I18" s="281"/>
+      <c r="H18" s="258"/>
+      <c r="I18" s="260"/>
     </row>
     <row r="19" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="I19" s="281"/>
+      <c r="I19" s="260"/>
     </row>
     <row r="20" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="I20" s="282"/>
+      <c r="I20" s="261"/>
     </row>
     <row r="23" spans="8:9" ht="14" x14ac:dyDescent="0.3">
       <c r="I23" s="50"/>
@@ -5454,35 +5454,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="256" t="s">
+      <c r="C1" s="282" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="256"/>
+      <c r="D1" s="282"/>
       <c r="E1" s="15"/>
       <c r="S1" s="77"/>
     </row>
     <row r="2" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="287" t="s">
+      <c r="A2" s="283" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="287"/>
-      <c r="C2" s="287"/>
-      <c r="D2" s="287"/>
-      <c r="E2" s="287"/>
-      <c r="F2" s="287"/>
-      <c r="G2" s="287"/>
-      <c r="H2" s="287"/>
-      <c r="I2" s="287"/>
-      <c r="J2" s="287"/>
-      <c r="K2" s="287"/>
-      <c r="L2" s="287"/>
-      <c r="M2" s="287"/>
-      <c r="N2" s="287"/>
-      <c r="O2" s="287"/>
-      <c r="P2" s="287"/>
-      <c r="Q2" s="287"/>
-      <c r="R2" s="287"/>
-      <c r="S2" s="287"/>
+      <c r="B2" s="283"/>
+      <c r="C2" s="283"/>
+      <c r="D2" s="283"/>
+      <c r="E2" s="283"/>
+      <c r="F2" s="283"/>
+      <c r="G2" s="283"/>
+      <c r="H2" s="283"/>
+      <c r="I2" s="283"/>
+      <c r="J2" s="283"/>
+      <c r="K2" s="283"/>
+      <c r="L2" s="283"/>
+      <c r="M2" s="283"/>
+      <c r="N2" s="283"/>
+      <c r="O2" s="283"/>
+      <c r="P2" s="283"/>
+      <c r="Q2" s="283"/>
+      <c r="R2" s="283"/>
+      <c r="S2" s="283"/>
     </row>
     <row r="3" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="78"/>
@@ -5591,7 +5591,7 @@
       <c r="B6" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="C6" s="257" t="str">
+      <c r="C6" s="284" t="str">
         <f>Greitis!C6</f>
         <v>XXXX</v>
       </c>
@@ -5671,7 +5671,7 @@
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="36"/>
       <c r="B7" s="33"/>
-      <c r="C7" s="258"/>
+      <c r="C7" s="285"/>
       <c r="D7" s="17"/>
       <c r="E7" s="18"/>
       <c r="F7" s="181">
@@ -5742,7 +5742,7 @@
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" s="36"/>
       <c r="B8" s="33"/>
-      <c r="C8" s="258"/>
+      <c r="C8" s="285"/>
       <c r="D8" s="17"/>
       <c r="E8" s="18"/>
       <c r="F8" s="181">
@@ -5813,7 +5813,7 @@
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="36"/>
       <c r="B9" s="33"/>
-      <c r="C9" s="258"/>
+      <c r="C9" s="285"/>
       <c r="D9" s="82"/>
       <c r="E9" s="82"/>
       <c r="F9" s="181">
@@ -5887,7 +5887,7 @@
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="82"/>
       <c r="B10" s="82"/>
-      <c r="C10" s="258"/>
+      <c r="C10" s="285"/>
       <c r="D10" s="82"/>
       <c r="E10" s="82"/>
       <c r="F10" s="181">
@@ -5937,13 +5937,13 @@
       </c>
       <c r="R10" s="82"/>
       <c r="S10" s="82"/>
-      <c r="T10" s="284" t="s">
+      <c r="T10" s="279" t="s">
         <v>30</v>
       </c>
-      <c r="U10" s="284" t="s">
+      <c r="U10" s="279" t="s">
         <v>31</v>
       </c>
-      <c r="V10" s="283" t="s">
+      <c r="V10" s="278" t="s">
         <v>35</v>
       </c>
       <c r="X10" s="232">
@@ -5958,7 +5958,7 @@
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="82"/>
       <c r="B11" s="82"/>
-      <c r="C11" s="258"/>
+      <c r="C11" s="285"/>
       <c r="D11" s="82"/>
       <c r="E11" s="82"/>
       <c r="F11" s="181">
@@ -6008,9 +6008,9 @@
       </c>
       <c r="R11" s="82"/>
       <c r="S11" s="82"/>
-      <c r="T11" s="285"/>
-      <c r="U11" s="285"/>
-      <c r="V11" s="283"/>
+      <c r="T11" s="280"/>
+      <c r="U11" s="280"/>
+      <c r="V11" s="278"/>
       <c r="X11" s="232">
         <f>Greitis!E11</f>
         <v>0.14000000000000001</v>
@@ -6023,7 +6023,7 @@
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" s="82"/>
       <c r="B12" s="82"/>
-      <c r="C12" s="258"/>
+      <c r="C12" s="285"/>
       <c r="D12" s="82"/>
       <c r="E12" s="82"/>
       <c r="F12" s="181">
@@ -6073,9 +6073,9 @@
       </c>
       <c r="R12" s="82"/>
       <c r="S12" s="82"/>
-      <c r="T12" s="286"/>
-      <c r="U12" s="286"/>
-      <c r="V12" s="283"/>
+      <c r="T12" s="281"/>
+      <c r="U12" s="281"/>
+      <c r="V12" s="278"/>
       <c r="X12" s="232">
         <f>Greitis!E12</f>
         <v>0.14000000000000001</v>
@@ -6088,7 +6088,7 @@
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="82"/>
       <c r="B13" s="82"/>
-      <c r="C13" s="258"/>
+      <c r="C13" s="285"/>
       <c r="D13" s="82"/>
       <c r="E13" s="82"/>
       <c r="F13" s="181">
@@ -6150,7 +6150,7 @@
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="82"/>
       <c r="B14" s="82"/>
-      <c r="C14" s="258"/>
+      <c r="C14" s="285"/>
       <c r="D14" s="82"/>
       <c r="E14" s="82"/>
       <c r="F14" s="181">
@@ -6212,7 +6212,7 @@
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="82"/>
       <c r="B15" s="82"/>
-      <c r="C15" s="258"/>
+      <c r="C15" s="285"/>
       <c r="D15" s="82"/>
       <c r="E15" s="82"/>
       <c r="F15" s="181">
@@ -6274,7 +6274,7 @@
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="82"/>
       <c r="B16" s="82"/>
-      <c r="C16" s="258"/>
+      <c r="C16" s="285"/>
       <c r="D16" s="82"/>
       <c r="E16" s="82"/>
       <c r="F16" s="181">
@@ -6336,7 +6336,7 @@
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" s="82"/>
       <c r="B17" s="82"/>
-      <c r="C17" s="258"/>
+      <c r="C17" s="285"/>
       <c r="D17" s="82"/>
       <c r="E17" s="82"/>
       <c r="F17" s="181">
@@ -6398,7 +6398,7 @@
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" s="82"/>
       <c r="B18" s="82"/>
-      <c r="C18" s="258"/>
+      <c r="C18" s="285"/>
       <c r="D18" s="82"/>
       <c r="E18" s="82"/>
       <c r="F18" s="181">
@@ -6460,7 +6460,7 @@
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" s="82"/>
       <c r="B19" s="82"/>
-      <c r="C19" s="258"/>
+      <c r="C19" s="285"/>
       <c r="D19" s="82"/>
       <c r="E19" s="82"/>
       <c r="F19" s="181">
@@ -6522,7 +6522,7 @@
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" s="82"/>
       <c r="B20" s="82"/>
-      <c r="C20" s="258"/>
+      <c r="C20" s="285"/>
       <c r="D20" s="82"/>
       <c r="E20" s="82"/>
       <c r="F20" s="181">
@@ -6584,7 +6584,7 @@
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" s="82"/>
       <c r="B21" s="82"/>
-      <c r="C21" s="258"/>
+      <c r="C21" s="285"/>
       <c r="D21" s="82"/>
       <c r="E21" s="82"/>
       <c r="F21" s="181">
@@ -6646,7 +6646,7 @@
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" s="83"/>
       <c r="B22" s="83"/>
-      <c r="C22" s="259"/>
+      <c r="C22" s="286"/>
       <c r="D22" s="83"/>
       <c r="E22" s="83"/>
       <c r="F22" s="181">
@@ -6792,26 +6792,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="256" t="s">
+      <c r="C1" s="282" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="256"/>
+      <c r="D1" s="282"/>
       <c r="Q1" s="16"/>
     </row>
     <row r="2" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="255" t="s">
+      <c r="C2" s="287" t="s">
         <v>95</v>
       </c>
-      <c r="D2" s="255"/>
-      <c r="E2" s="255"/>
-      <c r="F2" s="255"/>
-      <c r="G2" s="255"/>
-      <c r="H2" s="255"/>
-      <c r="I2" s="255"/>
-      <c r="J2" s="255"/>
-      <c r="K2" s="255"/>
-      <c r="L2" s="255"/>
-      <c r="M2" s="255"/>
+      <c r="D2" s="287"/>
+      <c r="E2" s="287"/>
+      <c r="F2" s="287"/>
+      <c r="G2" s="287"/>
+      <c r="H2" s="287"/>
+      <c r="I2" s="287"/>
+      <c r="J2" s="287"/>
+      <c r="K2" s="287"/>
+      <c r="L2" s="287"/>
+      <c r="M2" s="287"/>
       <c r="Q2" s="16"/>
     </row>
     <row r="3" spans="1:17" ht="12" customHeight="1" x14ac:dyDescent="0.3">
@@ -6873,7 +6873,7 @@
         <f>Paėmimas!B6</f>
         <v>XX</v>
       </c>
-      <c r="C6" s="257" t="str">
+      <c r="C6" s="284" t="str">
         <f>Paėmimas!C6</f>
         <v>XXXX</v>
       </c>
@@ -6925,7 +6925,7 @@
     <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="52"/>
       <c r="B7" s="21"/>
-      <c r="C7" s="258"/>
+      <c r="C7" s="285"/>
       <c r="D7" s="187">
         <f>Paėmimas!L7</f>
         <v>0.03</v>
@@ -6962,7 +6962,7 @@
     <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="52"/>
       <c r="B8" s="21"/>
-      <c r="C8" s="258"/>
+      <c r="C8" s="285"/>
       <c r="D8" s="187">
         <f>Paėmimas!L8</f>
         <v>0.03</v>
@@ -6999,7 +6999,7 @@
     <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="52"/>
       <c r="B9" s="21"/>
-      <c r="C9" s="258"/>
+      <c r="C9" s="285"/>
       <c r="D9" s="187">
         <f>Paėmimas!L9</f>
         <v>0.03</v>
@@ -7036,7 +7036,7 @@
     <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="52"/>
       <c r="B10" s="21"/>
-      <c r="C10" s="258"/>
+      <c r="C10" s="285"/>
       <c r="D10" s="187">
         <f>Paėmimas!L10</f>
         <v>0.03</v>
@@ -7073,7 +7073,7 @@
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="52"/>
       <c r="B11" s="21"/>
-      <c r="C11" s="258"/>
+      <c r="C11" s="285"/>
       <c r="D11" s="187">
         <f>Paėmimas!L11</f>
         <v>0.03</v>
@@ -7110,7 +7110,7 @@
     <row r="12" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="52"/>
       <c r="B12" s="21"/>
-      <c r="C12" s="258"/>
+      <c r="C12" s="285"/>
       <c r="D12" s="187">
         <f>Paėmimas!L12</f>
         <v>0.03</v>
@@ -7147,7 +7147,7 @@
     <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="52"/>
       <c r="B13" s="21"/>
-      <c r="C13" s="258"/>
+      <c r="C13" s="285"/>
       <c r="D13" s="187">
         <f>Paėmimas!L13</f>
         <v>0.03</v>
@@ -7184,7 +7184,7 @@
     <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="52"/>
       <c r="B14" s="21"/>
-      <c r="C14" s="258"/>
+      <c r="C14" s="285"/>
       <c r="D14" s="187">
         <f>Paėmimas!L14</f>
         <v>0.03</v>
@@ -7221,7 +7221,7 @@
     <row r="15" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="52"/>
       <c r="B15" s="21"/>
-      <c r="C15" s="258"/>
+      <c r="C15" s="285"/>
       <c r="D15" s="187">
         <f>Paėmimas!L15</f>
         <v>0.03</v>
@@ -7258,7 +7258,7 @@
     <row r="16" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="52"/>
       <c r="B16" s="21"/>
-      <c r="C16" s="258"/>
+      <c r="C16" s="285"/>
       <c r="D16" s="187">
         <f>Paėmimas!L16</f>
         <v>0.03</v>
@@ -7295,7 +7295,7 @@
     <row r="17" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="52"/>
       <c r="B17" s="21"/>
-      <c r="C17" s="258"/>
+      <c r="C17" s="285"/>
       <c r="D17" s="187">
         <f>Paėmimas!L17</f>
         <v>0.03</v>
@@ -7332,7 +7332,7 @@
     <row r="18" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="52"/>
       <c r="B18" s="21"/>
-      <c r="C18" s="258"/>
+      <c r="C18" s="285"/>
       <c r="D18" s="187">
         <f>Paėmimas!L18</f>
         <v>0.03</v>
@@ -7369,7 +7369,7 @@
     <row r="19" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="52"/>
       <c r="B19" s="21"/>
-      <c r="C19" s="258"/>
+      <c r="C19" s="285"/>
       <c r="D19" s="187">
         <f>Paėmimas!L19</f>
         <v>0.03</v>
@@ -7406,7 +7406,7 @@
     <row r="20" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="52"/>
       <c r="B20" s="21"/>
-      <c r="C20" s="258"/>
+      <c r="C20" s="285"/>
       <c r="D20" s="187">
         <f>Paėmimas!L20</f>
         <v>0.03</v>
@@ -7443,7 +7443,7 @@
     <row r="21" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="52"/>
       <c r="B21" s="21"/>
-      <c r="C21" s="258"/>
+      <c r="C21" s="285"/>
       <c r="D21" s="187">
         <f>Paėmimas!L21</f>
         <v>0.03</v>
@@ -7480,7 +7480,7 @@
     <row r="22" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="54"/>
       <c r="B22" s="55"/>
-      <c r="C22" s="259"/>
+      <c r="C22" s="286"/>
       <c r="D22" s="187">
         <f>Paėmimas!L22</f>
         <v>0.03</v>
@@ -7611,29 +7611,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="256" t="s">
+      <c r="C1" s="282" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="256"/>
+      <c r="D1" s="282"/>
       <c r="R1" s="16"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A2" s="255" t="s">
+      <c r="A2" s="287" t="s">
         <v>96</v>
       </c>
-      <c r="B2" s="255"/>
-      <c r="C2" s="255"/>
-      <c r="D2" s="255"/>
-      <c r="E2" s="255"/>
-      <c r="F2" s="255"/>
-      <c r="G2" s="255"/>
-      <c r="H2" s="255"/>
-      <c r="I2" s="255"/>
-      <c r="J2" s="255"/>
-      <c r="K2" s="255"/>
-      <c r="L2" s="255"/>
-      <c r="M2" s="255"/>
-      <c r="N2" s="255"/>
+      <c r="B2" s="287"/>
+      <c r="C2" s="287"/>
+      <c r="D2" s="287"/>
+      <c r="E2" s="287"/>
+      <c r="F2" s="287"/>
+      <c r="G2" s="287"/>
+      <c r="H2" s="287"/>
+      <c r="I2" s="287"/>
+      <c r="J2" s="287"/>
+      <c r="K2" s="287"/>
+      <c r="L2" s="287"/>
+      <c r="M2" s="287"/>
+      <c r="N2" s="287"/>
       <c r="O2" s="78"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
@@ -7837,31 +7837,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="256" t="s">
+      <c r="C1" s="282" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="256"/>
-      <c r="E1" s="256"/>
-      <c r="F1" s="256"/>
+      <c r="D1" s="282"/>
+      <c r="E1" s="282"/>
+      <c r="F1" s="282"/>
     </row>
     <row r="2" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="255" t="s">
+      <c r="A2" s="287" t="s">
         <v>97</v>
       </c>
-      <c r="B2" s="255"/>
-      <c r="C2" s="255"/>
-      <c r="D2" s="255"/>
-      <c r="E2" s="255"/>
-      <c r="F2" s="255"/>
-      <c r="G2" s="255"/>
-      <c r="H2" s="255"/>
-      <c r="I2" s="255"/>
-      <c r="J2" s="255"/>
-      <c r="K2" s="255"/>
-      <c r="L2" s="255"/>
-      <c r="M2" s="255"/>
-      <c r="N2" s="255"/>
-      <c r="O2" s="255"/>
+      <c r="B2" s="287"/>
+      <c r="C2" s="287"/>
+      <c r="D2" s="287"/>
+      <c r="E2" s="287"/>
+      <c r="F2" s="287"/>
+      <c r="G2" s="287"/>
+      <c r="H2" s="287"/>
+      <c r="I2" s="287"/>
+      <c r="J2" s="287"/>
+      <c r="K2" s="287"/>
+      <c r="L2" s="287"/>
+      <c r="M2" s="287"/>
+      <c r="N2" s="287"/>
+      <c r="O2" s="287"/>
       <c r="V2" s="16"/>
     </row>
     <row r="4" spans="1:22" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -8378,12 +8378,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8642,20 +8644,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8680,12 +8683,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{605DD0A7-BC00-4D8E-8AD3-26E2A9FDEA54}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
-    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>